<commit_message>
Lab 2: update deliverables to Problem Statement #35
Customizable Subscription Box Scheduler, Jira project SBOX.

- Product backlog: EPIC-1 Box Customization & Billing Cycle Control,
  6 user stories, 34 story points, sprints 18 / 16
- Sprint reflection answering the four lab questions
- Jira evidence: backlog, story points, active sprint board, burndown
- Lab 2 and root READMEs rewritten for PS #35
</commit_message>
<xml_diff>
--- a/Lab2/docs/01_Product_Backlog.xlsx
+++ b/Lab2/docs/01_Product_Backlog.xlsx
@@ -8,8 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprints" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epic &amp; Sprints" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -49,7 +48,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +58,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002F5C9E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4F7FC"/>
       </patternFill>
     </fill>
   </fills>
@@ -88,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -101,7 +105,18 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -467,184 +482,136 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Product Backlog - Campus Placement &amp; Internship Pipeline</t>
+          <t>Product Backlog - Customizable Subscription Box Scheduler</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prajwal G Devadiga | PES1UG24CS590 | Problem Statement #03 | Campus &amp; Academic Operations</t>
+          <t>Prajwal G Devadiga | PES1UG24CS590 | Problem Statement #35 | Retail, E-Commerce &amp; Finance</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>1 Epics | 6 User Stories | 34 points total | Sprint 1 = 21 | Sprint 2 = 13 | backlog = 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+          <t>1 Epic | 6 User Stories | 34 points | Sprint 1 = 18 | Sprint 2 = 16</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Scenario: A subscription box portal where subscribers customize monthly product selections (e.g. books, coffee, snacks) based on preference tags, with support for pausing or skipping billing cycles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Story ID</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Story Title</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>As a ...</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>I want to ...</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>So that ...</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Story Points</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Traces to</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K6" s="3" t="inlineStr">
         <is>
           <t>Planning Poker</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="46" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>EPIC-1 Drive Application &amp; Eligibility Screening</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
+    <row r="7" ht="52" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>EPIC-1 Box Customization &amp; Billing Cycle Control</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>US-1.1</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Upload &amp; Parse Resume</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>student applicant</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>upload my resume as a PDF and have my skill tags extracted from it automatically</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>I am matched to relevant drives without re-typing or tagging my own profile</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>CPIP Sprint 1</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>FR-001</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>Spread 5 / 8 / 13, settled at 8 - the upload itself is trivial; resumes have no fixed layout, so parsing accuracy is the real unknown rather than the coding effort.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="46" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>EPIC-1 Drive Application &amp; Eligibility Screening</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>US-1.2</t>
-        </is>
-      </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Create a Corporate Drive</t>
+          <t>Manage Preference Tags</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>placement officer</t>
+          <t>subscriber</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>create a drive with the role, CTC band and an application window</t>
+          <t>add or remove preference tags from the curated vocabulary on my profile</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>students can see the opportunity and apply to it</t>
+          <t>the box I am offered matches my tastes and avoids anything I cannot eat</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -657,7 +624,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>CPIP Sprint 1</t>
+          <t>SBOX Sprint 1</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -667,39 +634,39 @@
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>Spread 3 / 5, settled at 5 - the form is simple, but the window needs timezone-safe open and close handling and that is where the 3 was too optimistic.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="46" customHeight="1">
+          <t>Spread 3 / 5, settled at 5 - saving tags is trivial; treating exclusion tags such as nut-free as hard filters rather than ranking weights is what moved it off 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="52" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>EPIC-1 Drive Application &amp; Eligibility Screening</t>
+          <t>EPIC-1 Box Customization &amp; Billing Cycle Control</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>US-1.3</t>
+          <t>US-1.2</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Configure Multi-Tier Eligibility</t>
+          <t>Swap Items in the Next Box</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>placement officer</t>
+          <t>subscriber</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>set minimum CGPA, maximum active backlogs, permitted branches and a prior-offer cap on a drive</t>
+          <t>swap items in my upcoming box at any point up to 48 hours before renewal</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>ineligible students are screened out automatically instead of by hand</t>
+          <t>I receive a box I actually want instead of the default selection</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -712,49 +679,49 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>CPIP Sprint 1</t>
+          <t>SBOX Sprint 1</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>FR-002</t>
+          <t>FR-001</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>Spread 5 / 8 / 8, settled at 8 - four independent rule tiers that must compose, and each one has to stay individually explainable when it is the tier that fails.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="46" customHeight="1">
+          <t>Spread 5 / 8 / 13, settled at 8 - the swap itself is small, but re-picking a box whose stock is already reserved against the cycle is where the uncertainty sits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="52" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>EPIC-1 Drive Application &amp; Eligibility Screening</t>
+          <t>EPIC-1 Box Customization &amp; Billing Cycle Control</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>US-1.4</t>
+          <t>US-1.3</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>See Eligibility Status per Drive</t>
+          <t>Enforce the 48-Hour Cut-Off</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>student applicant</t>
+          <t>fulfillment lead</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>see whether I am eligible for each drive and exactly which rule I fail</t>
+          <t>have customization automatically refused once a box is inside 48 hours of renewal</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>I can contest a stale academic record instead of guessing why I was filtered out</t>
+          <t>the warehouse pick list stops moving underneath us</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -767,127 +734,182 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>CPIP Sprint 2</t>
+          <t>SBOX Sprint 1</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
+          <t>FR-001</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>Spread 3 / 5, settled at 5 - one server-side check, but it must read the renewal timestamp in UTC and never the browser clock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>EPIC-1 Box Customization &amp; Billing Cycle Control</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>US-1.4</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Pause or Skip a Billing Cycle</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>subscriber</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>pause a delivery or skip the next billing cycle without cancelling</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>I can take a break without losing my subscription and my preferences</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>SBOX Sprint 2</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
           <t>FR-001, FR-003</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>Spread 3 / 5, settled at 5 - rendering the list is easy; surfacing a per-tier reason for every failure is what makes the screen worth building.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="46" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>EPIC-1 Drive Application &amp; Eligibility Screening</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>Unanimous 5 - deferring the renewal date is simple; the three-skips-per-rolling-year cap is the only rule that has to be got right.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="52" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>EPIC-1 Box Customization &amp; Billing Cycle Control</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>US-1.5</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Apply to an Eligible Drive</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>student applicant</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>apply to a drive I am eligible for before its application window closes</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>I am considered by the visiting company</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Bill the Locked Box on Renewal</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>finance lead</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>have the system lock the box contents on the renewal date and charge the subscription, retrying a soft decline at most twice</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>revenue is collected without breaching card-scheme retry limits</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>CPIP Sprint 2</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>FR-003</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>Unanimous 5, and probably wrong - nobody raised that the submit path has to re-run the whole US-1.3 rule set at submission time, which makes it larger than it looked.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="46" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>EPIC-1 Drive Application &amp; Eligibility Screening</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="H11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>SBOX Sprint 2</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>FR-004</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>Spread 5 / 8 / 13, settled at 8 - bounded retries at 24-hour intervals plus the Suspended state are far more state than a single charge suggests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="52" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>EPIC-1 Box Customization &amp; Billing Cycle Control</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>US-1.6</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Enforce the Application Window</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>placement officer</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>late applications refused automatically with a clear reason code</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>the shortlist we hand the company is final and needs no manual reconciliation</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Generate the Fulfillment Manifest</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>fulfillment lead</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>generate the manifest for a cycle grouped by warehouse zone and export its shipping labels</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>the warehouse can pick and ship every paid box for that cycle</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H11" s="4" t="n">
+      <c r="H12" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>CPIP Sprint 2</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>FR-003</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>Spread 2 / 3, settled at 3 - one server-side check, but it must read server time and never the browser clock, which is what moved it off 2.</t>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>SBOX Sprint 2</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>FR-005, NFR-001</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>Unanimous 3, and wrong - nobody weighed NFR-001's 10,000 labels in under 60 seconds, which turns a list-generation story into a throughput problem.</t>
         </is>
       </c>
     </row>
@@ -902,308 +924,146 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>Traces to</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>Points</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>EPIC-1</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Drive Application &amp; Eligibility Screening</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Take a student from a published corporate drive to a submitted, screened application: publish the drive with its eligibility rule set, parse the student's resume, show them exactly where they stand against each rule, and let eligible students apply before the window closes.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>FR-001, FR-002, FR-003</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>Box Customization &amp; Billing Cycle Control</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>Take a subscriber from a personalised monthly box to a correctly billed and shipped one: capture preference tags, let them swap items or pause and skip a cycle before the 48-hour cut-off, then bill the locked box and hand the warehouse its manifest.</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>FR-001 to FR-005, NFR-001</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="n">
         <v>34</v>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>CPIP Sprint 1</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>21 pts</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>3 stories</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="9" t="n"/>
+      <c r="B3" s="9" t="n"/>
+      <c r="C3" s="9" t="n"/>
+      <c r="D3" s="9" t="n"/>
+      <c r="E3" s="9" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>Goal</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>A placement officer can publish a drive carrying its full eligibility rule set, and a student has a parsed profile for those rules to be evaluated against.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Story</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Why these items</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Stories</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>Points</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>US-1.1</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Upload &amp; Parse Resume</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>8</v>
-      </c>
-    </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>US-1.2</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Create a Corporate Drive</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>5</v>
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>SBOX Sprint 1</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>A subscriber can express their preferences and change the contents of their next box, with the 48-hour cut-off protecting the warehouse.</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 1 is the dependency root: preference tags have to exist before a box can be recommended, and a box has to be customisable before a cut-off means anything.</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>US-1.3</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Configure Multi-Tier Eligibility</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>CPIP Sprint 2</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>13 pts</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>3 stories</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Goal</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>A student can see exactly where they stand against every published drive and submit an application while the window is still open.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Story</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>US-1.4</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>See Eligibility Status per Drive</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>US-1.5</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Apply to an Eligible Drive</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>US-1.6</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Enforce the Application Window</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>SBOX Sprint 2</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>A subscriber can pause or skip a cycle, the locked box is billed on renewal, and the warehouse receives its manifest.</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 2 closes the loop from a customised box to a shipped one, consuming everything Sprint 1 produced.</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="n">
         <v>3</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>